<commit_message>
New tables and plots for thesis
</commit_message>
<xml_diff>
--- a/tables/Important/SpectraDetails.xlsx
+++ b/tables/Important/SpectraDetails.xlsx
@@ -425,86 +425,91 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q12"/>
+  <dimension ref="A1:R12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>id</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>OpticalID</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>T0</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Pobs</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>PHASE</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>ESO OBS TARG NAME</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>RA</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>DEC</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>DATE-OBS</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>MJD-OBS</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>WAVELMIN</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>WAVELMAX</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>SNR</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>SPEC_RES</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>TELESCOP</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>INSTRUME</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>file name</t>
         </is>
@@ -519,57 +524,62 @@
           <t>4U1538-52</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>QV Nor</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
         <v>52851.33</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>3.728414</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>0.006856081431919847</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>QV-Nor</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>235.597213</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>-52.38535</v>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>2010-04-11T04:41:00.641</t>
         </is>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>55297.19514631</v>
       </c>
-      <c r="K2" t="n">
-        <v>328.2031</v>
-      </c>
       <c r="L2" t="n">
-        <v>456.3057</v>
+        <v>3282.031</v>
       </c>
       <c r="M2" t="n">
+        <v>4563.057</v>
+      </c>
+      <c r="N2" t="n">
         <v>9.095800000000001</v>
       </c>
-      <c r="N2" t="n">
+      <c r="O2" t="n">
         <v>49620</v>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>ESO-VLT-U2</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>UVES</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>ADP.2020-06-19T07_46_26.470.fits</t>
         </is>
@@ -584,57 +594,62 @@
           <t>4U1538-52</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>QV Nor</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
         <v>52851.33</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>3.728414</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>0.006843974408070608</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>QV-Nor</t>
         </is>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>235.597213</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>-52.38535</v>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>2010-04-11T04:40:56.740</t>
         </is>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>55297.19510117</v>
       </c>
-      <c r="K3" t="n">
-        <v>458.3137</v>
-      </c>
       <c r="L3" t="n">
-        <v>668.6554</v>
+        <v>4583.137</v>
       </c>
       <c r="M3" t="n">
+        <v>6686.554</v>
+      </c>
+      <c r="N3" t="n">
         <v>63.7564</v>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>51690</v>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>ESO-VLT-U2</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>UVES</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>ADP.2020-06-19T07_46_26.479.fits</t>
         </is>
@@ -649,57 +664,62 @@
           <t>4U1700-37</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>HD 153919</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
         <v>48900.373</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>3.411581</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>0.001742910399116226</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>HD153919</t>
         </is>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>255.98644</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>-37.84445</v>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>2016-07-07T00:42:22.672</t>
         </is>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
         <v>57576.02942908</v>
       </c>
-      <c r="K4" t="n">
-        <v>304.423739693906</v>
-      </c>
       <c r="L4" t="n">
-        <v>391.666842081719</v>
+        <v>3044.23739693906</v>
       </c>
       <c r="M4" t="n">
+        <v>3916.66842081719</v>
+      </c>
+      <c r="N4" t="n">
         <v>116.186873803252</v>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>71050</v>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>ESO-VLT-U2</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>UVES</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>ADP.2020-06-10T08_35_48.825.fits</t>
         </is>
@@ -714,57 +734,62 @@
           <t>4U1700-37</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>HD 153919</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
         <v>48900.373</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>3.411581</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>0.001729423102915462</v>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>HD153919</t>
         </is>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>255.98644</v>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>-37.84445</v>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>2016-07-07T00:42:18.696</t>
         </is>
       </c>
-      <c r="J5" t="n">
+      <c r="K5" t="n">
         <v>57576.029383067</v>
       </c>
-      <c r="K5" t="n">
-        <v>458.309103563039</v>
-      </c>
       <c r="L5" t="n">
-        <v>668.647357735182</v>
+        <v>4583.09103563039</v>
       </c>
       <c r="M5" t="n">
+        <v>6686.47357735182</v>
+      </c>
+      <c r="N5" t="n">
         <v>330.342469438816</v>
       </c>
-      <c r="N5" t="n">
+      <c r="O5" t="n">
         <v>107200</v>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>ESO-VLT-U2</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>UVES</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>ADP.2020-06-10T08_35_48.989.fits</t>
         </is>
@@ -779,57 +804,62 @@
           <t>Cen X-3</t>
         </is>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>V779 Cen</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
         <v>50506.788423</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>2.08704106</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>0.7398526505276095</v>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Cen-X-3</t>
         </is>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
         <v>170.314352</v>
       </c>
-      <c r="H6" t="n">
+      <c r="I6" t="n">
         <v>-60.6237</v>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>2002-02-23T05:34:33.327</t>
         </is>
       </c>
-      <c r="J6" t="n">
+      <c r="K6" t="n">
         <v>52328.23233018</v>
       </c>
-      <c r="K6" t="n">
-        <v>458.3455</v>
-      </c>
       <c r="L6" t="n">
-        <v>668.6468</v>
+        <v>4583.455</v>
       </c>
       <c r="M6" t="n">
+        <v>6686.468</v>
+      </c>
+      <c r="N6" t="n">
         <v>90.71169999999999</v>
       </c>
-      <c r="N6" t="n">
+      <c r="O6" t="n">
         <v>42310</v>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>ESO-VLT-U2</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>UVES</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="R6" t="inlineStr">
         <is>
           <t>ADP.2021-08-26T17_28_27.478.fits</t>
         </is>
@@ -844,57 +874,62 @@
           <t>Cen X-3</t>
         </is>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>V779 Cen</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
         <v>50506.788423</v>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
         <v>2.08704106</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>0.7398562872564298</v>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Cen-X-3</t>
         </is>
       </c>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
         <v>170.314352</v>
       </c>
-      <c r="H7" t="n">
+      <c r="I7" t="n">
         <v>-60.6237</v>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>2002-02-23T05:34:33.983</t>
         </is>
       </c>
-      <c r="J7" t="n">
+      <c r="K7" t="n">
         <v>52328.23233777</v>
       </c>
-      <c r="K7" t="n">
-        <v>328.1074</v>
-      </c>
       <c r="L7" t="n">
-        <v>456.2458</v>
+        <v>3281.074</v>
       </c>
       <c r="M7" t="n">
+        <v>4562.458</v>
+      </c>
+      <c r="N7" t="n">
         <v>32.8209</v>
       </c>
-      <c r="N7" t="n">
+      <c r="O7" t="n">
         <v>40970</v>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>ESO-VLT-U2</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>UVES</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr">
+      <c r="R7" t="inlineStr">
         <is>
           <t>ADP.2021-08-26T17_28_27.490.fits</t>
         </is>
@@ -909,57 +944,62 @@
           <t>LMC X-4</t>
         </is>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>LMC X-4</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
         <v>51110.86579</v>
       </c>
-      <c r="D8" t="n">
+      <c r="E8" t="n">
         <v>1.408379</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>0.4193713907935717</v>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>LMC-X-4</t>
         </is>
       </c>
-      <c r="G8" t="n">
+      <c r="H8" t="n">
         <v>83.20695600000001</v>
       </c>
-      <c r="H8" t="n">
+      <c r="I8" t="n">
         <v>-66.37112</v>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>2001-12-02T04:50:11.229</t>
         </is>
       </c>
-      <c r="J8" t="n">
+      <c r="K8" t="n">
         <v>52245.20151886</v>
       </c>
-      <c r="K8" t="n">
-        <v>328.1097</v>
-      </c>
       <c r="L8" t="n">
-        <v>456.2446</v>
+        <v>3281.097</v>
       </c>
       <c r="M8" t="n">
+        <v>4562.446</v>
+      </c>
+      <c r="N8" t="n">
         <v>59.5739</v>
       </c>
-      <c r="N8" t="n">
+      <c r="O8" t="n">
         <v>40970</v>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>ESO-VLT-U2</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>UVES</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr">
+      <c r="R8" t="inlineStr">
         <is>
           <t>ADP.2021-09-09T09_02_25.134.fits</t>
         </is>
@@ -974,57 +1014,62 @@
           <t>LMC X-4</t>
         </is>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>LMC X-4</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
         <v>51110.86579</v>
       </c>
-      <c r="D9" t="n">
+      <c r="E9" t="n">
         <v>1.408379</v>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>0.4201579617417792</v>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>LMC-X-4</t>
         </is>
       </c>
-      <c r="G9" t="n">
+      <c r="H9" t="n">
         <v>83.20695600000001</v>
       </c>
-      <c r="H9" t="n">
+      <c r="I9" t="n">
         <v>-66.37112</v>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>2001-12-02T04:51:46.942</t>
         </is>
       </c>
-      <c r="J9" t="n">
+      <c r="K9" t="n">
         <v>52245.20262665</v>
       </c>
-      <c r="K9" t="n">
-        <v>458.3488</v>
-      </c>
       <c r="L9" t="n">
-        <v>668.649</v>
+        <v>4583.487999999999</v>
       </c>
       <c r="M9" t="n">
+        <v>6686.49</v>
+      </c>
+      <c r="N9" t="n">
         <v>64.8361</v>
       </c>
-      <c r="N9" t="n">
+      <c r="O9" t="n">
         <v>42310</v>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="P9" t="inlineStr">
         <is>
           <t>ESO-VLT-U2</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>UVES</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr">
+      <c r="R9" t="inlineStr">
         <is>
           <t>ADP.2021-09-09T09_02_25.907.fits</t>
         </is>
@@ -1039,57 +1084,62 @@
           <t>SMC X-1</t>
         </is>
       </c>
-      <c r="C10" t="n">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Sk 160</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
         <v>50324.691861</v>
       </c>
-      <c r="D10" t="n">
+      <c r="E10" t="n">
         <v>3.89192316</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>0.5434266204783853</v>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>SMC-X-1</t>
         </is>
       </c>
-      <c r="G10" t="n">
+      <c r="H10" t="n">
         <v>19.271752</v>
       </c>
-      <c r="H10" t="n">
+      <c r="I10" t="n">
         <v>-73.44356999999999</v>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>2001-10-05T03:30:23.569</t>
         </is>
       </c>
-      <c r="J10" t="n">
+      <c r="K10" t="n">
         <v>52187.14610613</v>
       </c>
-      <c r="K10" t="n">
-        <v>328.1079</v>
-      </c>
       <c r="L10" t="n">
-        <v>456.2432</v>
+        <v>3281.079</v>
       </c>
       <c r="M10" t="n">
+        <v>4562.432</v>
+      </c>
+      <c r="N10" t="n">
         <v>50.2435</v>
       </c>
-      <c r="N10" t="n">
+      <c r="O10" t="n">
         <v>40970</v>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>ESO-VLT-U2</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="Q10" t="inlineStr">
         <is>
           <t>UVES</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr">
+      <c r="R10" t="inlineStr">
         <is>
           <t>ADP.2020-08-14T14_51_21.171.fits</t>
         </is>
@@ -1104,57 +1154,62 @@
           <t>SMC X-1</t>
         </is>
       </c>
-      <c r="C11" t="n">
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Sk 160</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
         <v>50324.691861</v>
       </c>
-      <c r="D11" t="n">
+      <c r="E11" t="n">
         <v>3.89192316</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>0.5437749264308422</v>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>SMC-X-1</t>
         </is>
       </c>
-      <c r="G11" t="n">
+      <c r="H11" t="n">
         <v>19.271752</v>
       </c>
-      <c r="H11" t="n">
+      <c r="I11" t="n">
         <v>-73.44356999999999</v>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>2001-10-05T03:32:20.691</t>
         </is>
       </c>
-      <c r="J11" t="n">
+      <c r="K11" t="n">
         <v>52187.14746171</v>
       </c>
-      <c r="K11" t="n">
-        <v>458.3488</v>
-      </c>
       <c r="L11" t="n">
-        <v>668.6489</v>
+        <v>4583.487999999999</v>
       </c>
       <c r="M11" t="n">
+        <v>6686.489</v>
+      </c>
+      <c r="N11" t="n">
         <v>69.8227</v>
       </c>
-      <c r="N11" t="n">
+      <c r="O11" t="n">
         <v>42310</v>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="P11" t="inlineStr">
         <is>
           <t>ESO-VLT-U2</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="Q11" t="inlineStr">
         <is>
           <t>UVES</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr">
+      <c r="R11" t="inlineStr">
         <is>
           <t>ADP.2020-08-14T14_51_21.178.fits</t>
         </is>
@@ -1169,57 +1224,62 @@
           <t>Vela X-1</t>
         </is>
       </c>
-      <c r="C12" t="n">
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>HD 77581</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
         <v>48895.2186</v>
       </c>
-      <c r="D12" t="n">
+      <c r="E12" t="n">
         <v>8.964427000000001</v>
       </c>
-      <c r="E12" t="n">
+      <c r="F12" t="n">
         <v>0.4403336186462639</v>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>GP Vel</t>
         </is>
       </c>
-      <c r="G12" t="n">
+      <c r="H12" t="n">
         <v>135.513366</v>
       </c>
-      <c r="H12" t="n">
+      <c r="I12" t="n">
         <v>-40.54151</v>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>2022-12-21T09:00:49.730</t>
         </is>
       </c>
-      <c r="J12" t="n">
+      <c r="K12" t="n">
         <v>59934.37557558</v>
       </c>
-      <c r="K12" t="n">
-        <v>352.7789999966</v>
-      </c>
       <c r="L12" t="n">
-        <v>921.7319872796</v>
+        <v>3527.789999966</v>
       </c>
       <c r="M12" t="n">
+        <v>9217.319872796001</v>
+      </c>
+      <c r="N12" t="n">
         <v>377.9</v>
       </c>
-      <c r="N12" t="n">
+      <c r="O12" t="n">
         <v>48000</v>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="P12" t="inlineStr">
         <is>
           <t>MPG/ESO-2.2</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
+      <c r="Q12" t="inlineStr">
         <is>
           <t>FEROS</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr">
+      <c r="R12" t="inlineStr">
         <is>
           <t>ADP.2023-01-09T23_22_13.954.fits</t>
         </is>

</xml_diff>